<commit_message>
Deploying to gh-pages from  @ a5d40efbdf7813c90404cddd4ab48fd4fb7c0585 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/16.1.1.xlsx
+++ b/en/downloads/data-excel/16.1.1.xlsx
@@ -1,15 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43A5CEC-ED0A-4FA8-828A-56F8E22A24E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -283,7 +295,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -471,19 +483,13 @@
   </cellStyleXfs>
   <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -493,7 +499,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -502,73 +508,50 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -577,9 +560,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -590,11 +570,31 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 6" xfId="1"/>
+    <cellStyle name="Обычный 6" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -610,9 +610,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -650,9 +650,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -687,7 +687,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -722,7 +722,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -895,7 +895,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -905,66 +905,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-    </row>
-    <row r="2" spans="1:17" s="38" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+    </row>
+    <row r="2" spans="1:17" s="27" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
-      <c r="N2" s="37"/>
-      <c r="O2" s="37"/>
-      <c r="P2" s="37"/>
-      <c r="Q2" s="37"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
     </row>
     <row r="3" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="39"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
     </row>
     <row r="4" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -973,1715 +974,1796 @@
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>2014</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <v>2015</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>2016</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>2017</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>2018</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>2019</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>2020</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>2021</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>2022</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="3">
         <v>2023</v>
       </c>
-      <c r="N4" s="40">
+      <c r="N4" s="29">
         <v>2024</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" s="6" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="O4" s="29">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" s="40" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="38">
         <v>5.3588234703070938</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="38">
         <v>4.9929517528616572</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="38">
         <v>4.2774313111816866</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="38">
         <v>4.0180012735180597</v>
       </c>
-      <c r="H5" s="26">
+      <c r="H5" s="38">
         <v>3.1150114396109765</v>
       </c>
-      <c r="I5" s="26">
+      <c r="I5" s="38">
         <v>2.6112042874173569</v>
       </c>
-      <c r="J5" s="26">
+      <c r="J5" s="38">
         <v>2.5332865755400285</v>
       </c>
-      <c r="K5" s="26">
+      <c r="K5" s="38">
         <v>2.6327784680382864</v>
       </c>
-      <c r="L5" s="26">
+      <c r="L5" s="38">
         <v>2.713997263267681</v>
       </c>
-      <c r="M5" s="26">
+      <c r="M5" s="38">
         <v>1.4800521090044416</v>
       </c>
-      <c r="N5" s="41">
+      <c r="N5" s="39">
         <f>N6/N7*100000</f>
         <v>1.4419458193664858</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" s="6" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="O5" s="39">
+        <f>O6/O7*100000</f>
+        <v>1.5261342384975058</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="40" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="42">
         <v>320</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="42">
         <v>305</v>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="42">
         <v>267</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="42">
         <v>256</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="42">
         <v>203</v>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="42">
         <v>174</v>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="42">
         <v>172</v>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="42">
         <v>182</v>
       </c>
-      <c r="L6" s="27">
+      <c r="L6" s="42">
         <v>191</v>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="42">
         <v>106</v>
       </c>
-      <c r="N6" s="42">
+      <c r="N6" s="43">
         <v>105</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" s="6" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="O6" s="43">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" s="40" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="45" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="46">
         <v>5971460</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="46">
         <v>6108611</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="46">
         <v>6242064</v>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="46">
         <v>6371327</v>
       </c>
-      <c r="H7" s="28">
+      <c r="H7" s="46">
         <v>6516830</v>
       </c>
-      <c r="I7" s="28">
+      <c r="I7" s="46">
         <v>6663592</v>
       </c>
-      <c r="J7" s="28">
+      <c r="J7" s="46">
         <v>6789599</v>
       </c>
-      <c r="K7" s="28">
+      <c r="K7" s="46">
         <v>6912849</v>
       </c>
-      <c r="L7" s="28">
+      <c r="L7" s="46">
         <v>7037590</v>
       </c>
-      <c r="M7" s="28">
+      <c r="M7" s="46">
         <v>7161910</v>
       </c>
-      <c r="N7" s="43">
+      <c r="N7" s="47">
         <v>7281827</v>
       </c>
+      <c r="O7" s="48">
+        <v>7404329</v>
+      </c>
     </row>
     <row r="8" spans="1:17" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="28"/>
-      <c r="M8" s="28"/>
-      <c r="N8" s="43"/>
-    </row>
-    <row r="9" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="36"/>
+      <c r="O8" s="31"/>
+    </row>
+    <row r="9" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="20">
         <v>7.6306080305875472</v>
       </c>
-      <c r="E9" s="28">
+      <c r="E9" s="20">
         <v>7.4887651954004406</v>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="20">
         <v>6.5483426533754763</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="20">
         <v>6.160026697682718</v>
       </c>
-      <c r="H9" s="28">
+      <c r="H9" s="20">
         <v>5.0272557948432768</v>
       </c>
-      <c r="I9" s="28">
+      <c r="I9" s="20">
         <v>3.9748932392224261</v>
       </c>
-      <c r="J9" s="28">
+      <c r="J9" s="20">
         <v>4.0208560313138317</v>
       </c>
-      <c r="K9" s="28">
+      <c r="K9" s="20">
         <v>4.213793854181664</v>
       </c>
-      <c r="L9" s="28">
+      <c r="L9" s="20">
         <v>4.2525094115503901</v>
       </c>
-      <c r="M9" s="28">
+      <c r="M9" s="20">
         <v>2.3991814557386304</v>
       </c>
-      <c r="N9" s="43">
+      <c r="N9" s="31">
         <v>2.2000000000000002</v>
       </c>
+      <c r="O9" s="31">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="20">
         <v>3.1427721698592266</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="20">
         <v>2.5560081235761984</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="20">
         <v>2.0587119304573442</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="20">
         <v>1.9242766116592542</v>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="20">
         <v>1.2445376937077388</v>
       </c>
-      <c r="I10" s="28">
+      <c r="I10" s="20">
         <v>1.2767577242357713</v>
       </c>
-      <c r="J10" s="28">
+      <c r="J10" s="20">
         <v>1.0780555956184326</v>
       </c>
-      <c r="K10" s="28">
+      <c r="K10" s="20">
         <v>1.0871116901411273</v>
       </c>
-      <c r="L10" s="28">
+      <c r="L10" s="20">
         <v>1.2087846597917742</v>
       </c>
-      <c r="M10" s="28">
+      <c r="M10" s="20">
         <v>0.5802651811878029</v>
       </c>
-      <c r="N10" s="43">
+      <c r="N10" s="31">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" s="21" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
+      <c r="O10" s="31">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" s="15" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
-      <c r="M11" s="29"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="48"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="30"/>
+      <c r="O11" s="30"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="20">
         <v>225</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="20">
         <v>226</v>
       </c>
-      <c r="F12" s="28">
+      <c r="F12" s="20">
         <v>202</v>
       </c>
-      <c r="G12" s="28">
+      <c r="G12" s="20">
         <v>194</v>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="20">
         <v>162</v>
       </c>
-      <c r="I12" s="28">
+      <c r="I12" s="20">
         <v>131</v>
       </c>
-      <c r="J12" s="28">
+      <c r="J12" s="20">
         <v>135</v>
       </c>
-      <c r="K12" s="28">
+      <c r="K12" s="20">
         <v>144</v>
       </c>
-      <c r="L12" s="28">
+      <c r="L12" s="20">
         <v>148</v>
       </c>
-      <c r="M12" s="28">
+      <c r="M12" s="20">
         <v>85</v>
       </c>
-      <c r="N12" s="43">
+      <c r="N12" s="31">
         <v>80</v>
       </c>
+      <c r="O12" s="31">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="20">
         <v>95</v>
       </c>
-      <c r="E13" s="28">
+      <c r="E13" s="20">
         <v>79</v>
       </c>
-      <c r="F13" s="28">
+      <c r="F13" s="20">
         <v>65</v>
       </c>
-      <c r="G13" s="28">
+      <c r="G13" s="20">
         <v>62</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="20">
         <v>41</v>
       </c>
-      <c r="I13" s="28">
+      <c r="I13" s="20">
         <v>43</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="20">
         <v>37</v>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="20">
         <v>38</v>
       </c>
-      <c r="L13" s="28">
+      <c r="L13" s="20">
         <v>43</v>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="20">
         <v>21</v>
       </c>
-      <c r="N13" s="43">
+      <c r="N13" s="31">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="O13" s="31">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="28"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="43"/>
-    </row>
-    <row r="15" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="20"/>
+      <c r="M14" s="20"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="31"/>
+    </row>
+    <row r="15" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="27">
+      <c r="D15" s="19">
         <v>12</v>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="19">
         <v>13</v>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="19">
         <v>11</v>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="19">
         <v>6</v>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="19">
         <v>13</v>
       </c>
-      <c r="I15" s="27">
+      <c r="I15" s="19">
         <v>21</v>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="19">
         <v>19</v>
       </c>
-      <c r="K15" s="27">
+      <c r="K15" s="19">
         <v>14</v>
       </c>
-      <c r="L15" s="27">
+      <c r="L15" s="19">
         <v>8</v>
       </c>
-      <c r="M15" s="27">
+      <c r="M15" s="19">
         <v>7</v>
       </c>
-      <c r="N15" s="44">
+      <c r="N15" s="32">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="O15" s="32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="20">
         <v>12</v>
       </c>
-      <c r="E16" s="28">
+      <c r="E16" s="20">
         <v>11</v>
       </c>
-      <c r="F16" s="28">
+      <c r="F16" s="20">
         <v>9</v>
       </c>
-      <c r="G16" s="28">
+      <c r="G16" s="20">
         <v>4</v>
       </c>
-      <c r="H16" s="28">
+      <c r="H16" s="20">
         <v>10</v>
       </c>
-      <c r="I16" s="28">
+      <c r="I16" s="20">
         <v>18</v>
       </c>
-      <c r="J16" s="28">
+      <c r="J16" s="20">
         <v>16</v>
       </c>
-      <c r="K16" s="28">
+      <c r="K16" s="20">
         <v>12</v>
       </c>
-      <c r="L16" s="28">
+      <c r="L16" s="20">
         <v>5</v>
       </c>
-      <c r="M16" s="28"/>
-      <c r="N16" s="45"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="M16" s="20"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D17" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="28">
+      <c r="E17" s="20">
         <v>2</v>
       </c>
-      <c r="F17" s="28">
+      <c r="F17" s="20">
         <v>2</v>
       </c>
-      <c r="G17" s="28">
+      <c r="G17" s="20">
         <v>2</v>
       </c>
-      <c r="H17" s="28">
+      <c r="H17" s="20">
         <v>3</v>
       </c>
-      <c r="I17" s="28">
+      <c r="I17" s="20">
         <v>3</v>
       </c>
-      <c r="J17" s="28">
+      <c r="J17" s="20">
         <v>3</v>
       </c>
-      <c r="K17" s="28">
+      <c r="K17" s="20">
         <v>2</v>
       </c>
-      <c r="L17" s="28">
+      <c r="L17" s="20">
         <v>3</v>
       </c>
-      <c r="M17" s="28"/>
-      <c r="N17" s="45"/>
-    </row>
-    <row r="18" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="M17" s="20"/>
+      <c r="N17" s="33"/>
+      <c r="O17" s="33"/>
+    </row>
+    <row r="18" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="19">
         <v>39</v>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="19">
         <v>43</v>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="19">
         <v>30</v>
       </c>
-      <c r="G18" s="27">
+      <c r="G18" s="19">
         <v>20</v>
       </c>
-      <c r="H18" s="27">
+      <c r="H18" s="19">
         <v>19</v>
       </c>
-      <c r="I18" s="27">
+      <c r="I18" s="19">
         <v>21</v>
       </c>
-      <c r="J18" s="27">
+      <c r="J18" s="19">
         <v>31</v>
       </c>
-      <c r="K18" s="27">
+      <c r="K18" s="19">
         <v>16</v>
       </c>
-      <c r="L18" s="27">
+      <c r="L18" s="19">
         <v>18</v>
       </c>
-      <c r="M18" s="27">
+      <c r="M18" s="19">
         <v>11</v>
       </c>
-      <c r="N18" s="44">
+      <c r="N18" s="32">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="O18" s="32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="20">
         <v>29</v>
       </c>
-      <c r="E19" s="28">
+      <c r="E19" s="20">
         <v>31</v>
       </c>
-      <c r="F19" s="28">
+      <c r="F19" s="20">
         <v>22</v>
       </c>
-      <c r="G19" s="28">
+      <c r="G19" s="20">
         <v>12</v>
       </c>
-      <c r="H19" s="28">
+      <c r="H19" s="20">
         <v>17</v>
       </c>
-      <c r="I19" s="28">
+      <c r="I19" s="20">
         <v>16</v>
       </c>
-      <c r="J19" s="28">
+      <c r="J19" s="20">
         <v>23</v>
       </c>
-      <c r="K19" s="28">
+      <c r="K19" s="20">
         <v>13</v>
       </c>
-      <c r="L19" s="28">
+      <c r="L19" s="20">
         <v>13</v>
       </c>
-      <c r="M19" s="28"/>
-      <c r="N19" s="45"/>
-    </row>
-    <row r="20" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="M19" s="20"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+    </row>
+    <row r="20" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="20">
         <v>10</v>
       </c>
-      <c r="E20" s="28">
+      <c r="E20" s="20">
         <v>12</v>
       </c>
-      <c r="F20" s="28">
+      <c r="F20" s="20">
         <v>8</v>
       </c>
-      <c r="G20" s="28">
+      <c r="G20" s="20">
         <v>8</v>
       </c>
-      <c r="H20" s="28">
+      <c r="H20" s="20">
         <v>2</v>
       </c>
-      <c r="I20" s="28">
+      <c r="I20" s="20">
         <v>5</v>
       </c>
-      <c r="J20" s="28">
+      <c r="J20" s="20">
         <v>8</v>
       </c>
-      <c r="K20" s="28">
+      <c r="K20" s="20">
         <v>3</v>
       </c>
-      <c r="L20" s="28">
+      <c r="L20" s="20">
         <v>5</v>
       </c>
-      <c r="M20" s="28"/>
-      <c r="N20" s="45"/>
-    </row>
-    <row r="21" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
+      <c r="M20" s="20"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+    </row>
+    <row r="21" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="27">
+      <c r="D21" s="19">
         <v>31</v>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="19">
         <v>28</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="19">
         <v>27</v>
       </c>
-      <c r="G21" s="27">
+      <c r="G21" s="19">
         <v>23</v>
       </c>
-      <c r="H21" s="27">
+      <c r="H21" s="19">
         <v>15</v>
       </c>
-      <c r="I21" s="27">
+      <c r="I21" s="19">
         <v>18</v>
       </c>
-      <c r="J21" s="27">
+      <c r="J21" s="19">
         <v>12</v>
       </c>
-      <c r="K21" s="27">
+      <c r="K21" s="19">
         <v>11</v>
       </c>
-      <c r="L21" s="27">
+      <c r="L21" s="19">
         <v>14</v>
       </c>
-      <c r="M21" s="27">
+      <c r="M21" s="19">
         <v>10</v>
       </c>
-      <c r="N21" s="44">
+      <c r="N21" s="32">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+      <c r="O21" s="32">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="20">
         <v>17</v>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="20">
         <v>19</v>
       </c>
-      <c r="F22" s="28">
+      <c r="F22" s="20">
         <v>20</v>
       </c>
-      <c r="G22" s="28">
+      <c r="G22" s="20">
         <v>17</v>
       </c>
-      <c r="H22" s="28">
+      <c r="H22" s="20">
         <v>14</v>
       </c>
-      <c r="I22" s="28">
+      <c r="I22" s="20">
         <v>15</v>
       </c>
-      <c r="J22" s="28">
+      <c r="J22" s="20">
         <v>9</v>
       </c>
-      <c r="K22" s="28">
+      <c r="K22" s="20">
         <v>8</v>
       </c>
-      <c r="L22" s="28">
+      <c r="L22" s="20">
         <v>10</v>
       </c>
-      <c r="M22" s="28"/>
-      <c r="N22" s="45"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="M22" s="20"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="20">
         <v>14</v>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="20">
         <v>9</v>
       </c>
-      <c r="F23" s="28">
+      <c r="F23" s="20">
         <v>7</v>
       </c>
-      <c r="G23" s="28">
+      <c r="G23" s="20">
         <v>6</v>
       </c>
-      <c r="H23" s="28">
+      <c r="H23" s="20">
         <v>1</v>
       </c>
-      <c r="I23" s="28">
+      <c r="I23" s="20">
         <v>3</v>
       </c>
-      <c r="J23" s="28">
+      <c r="J23" s="20">
         <v>3</v>
       </c>
-      <c r="K23" s="28">
+      <c r="K23" s="20">
         <v>3</v>
       </c>
-      <c r="L23" s="28">
+      <c r="L23" s="20">
         <v>4</v>
       </c>
-      <c r="M23" s="28"/>
-      <c r="N23" s="45"/>
-    </row>
-    <row r="24" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17" t="s">
+      <c r="M23" s="20"/>
+      <c r="N23" s="33"/>
+      <c r="O23" s="33"/>
+    </row>
+    <row r="24" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="27">
+      <c r="D24" s="19">
         <v>14</v>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="19">
         <v>11</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="19">
         <v>6</v>
       </c>
-      <c r="G24" s="27">
+      <c r="G24" s="19">
         <v>6</v>
       </c>
-      <c r="H24" s="27">
+      <c r="H24" s="19">
         <v>5</v>
       </c>
-      <c r="I24" s="27">
+      <c r="I24" s="19">
         <v>5</v>
       </c>
-      <c r="J24" s="27">
+      <c r="J24" s="19">
         <v>7</v>
       </c>
-      <c r="K24" s="27">
+      <c r="K24" s="19">
         <v>7</v>
       </c>
-      <c r="L24" s="27">
+      <c r="L24" s="19">
         <v>10</v>
       </c>
-      <c r="M24" s="27">
+      <c r="M24" s="19">
         <v>2</v>
       </c>
-      <c r="N24" s="44">
+      <c r="N24" s="32">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+      <c r="O24" s="32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="20">
         <v>14</v>
       </c>
-      <c r="E25" s="28">
+      <c r="E25" s="20">
         <v>7</v>
       </c>
-      <c r="F25" s="28">
+      <c r="F25" s="20">
         <v>4</v>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="20">
         <v>4</v>
       </c>
-      <c r="H25" s="28">
+      <c r="H25" s="20">
         <v>3</v>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="20">
         <v>4</v>
       </c>
-      <c r="J25" s="28">
+      <c r="J25" s="20">
         <v>4</v>
       </c>
-      <c r="K25" s="28">
+      <c r="K25" s="20">
         <v>4</v>
       </c>
-      <c r="L25" s="28">
+      <c r="L25" s="20">
         <v>8</v>
       </c>
-      <c r="M25" s="28"/>
-      <c r="N25" s="45"/>
-    </row>
-    <row r="26" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
+      <c r="M25" s="20"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="33"/>
+    </row>
+    <row r="26" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="30" t="s">
+      <c r="D26" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="28">
+      <c r="E26" s="20">
         <v>4</v>
       </c>
-      <c r="F26" s="28">
+      <c r="F26" s="20">
         <v>2</v>
       </c>
-      <c r="G26" s="28">
+      <c r="G26" s="20">
         <v>2</v>
       </c>
-      <c r="H26" s="28">
+      <c r="H26" s="20">
         <v>2</v>
       </c>
-      <c r="I26" s="28">
+      <c r="I26" s="20">
         <v>1</v>
       </c>
-      <c r="J26" s="28">
+      <c r="J26" s="20">
         <v>3</v>
       </c>
-      <c r="K26" s="28">
+      <c r="K26" s="20">
         <v>3</v>
       </c>
-      <c r="L26" s="28">
+      <c r="L26" s="20">
         <v>2</v>
       </c>
-      <c r="M26" s="28"/>
-      <c r="N26" s="45"/>
-    </row>
-    <row r="27" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="18" t="s">
+      <c r="M26" s="20"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="33"/>
+    </row>
+    <row r="27" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="27">
+      <c r="D27" s="19">
         <v>16</v>
       </c>
-      <c r="E27" s="27">
+      <c r="E27" s="19">
         <v>24</v>
       </c>
-      <c r="F27" s="27">
+      <c r="F27" s="19">
         <v>22</v>
       </c>
-      <c r="G27" s="27">
+      <c r="G27" s="19">
         <v>12</v>
       </c>
-      <c r="H27" s="27">
+      <c r="H27" s="19">
         <v>14</v>
       </c>
-      <c r="I27" s="27">
+      <c r="I27" s="19">
         <v>15</v>
       </c>
-      <c r="J27" s="27">
+      <c r="J27" s="19">
         <v>11</v>
       </c>
-      <c r="K27" s="27">
+      <c r="K27" s="19">
         <v>24</v>
       </c>
-      <c r="L27" s="27">
+      <c r="L27" s="19">
         <v>19</v>
       </c>
-      <c r="M27" s="27">
+      <c r="M27" s="19">
         <v>9</v>
       </c>
-      <c r="N27" s="44">
+      <c r="N27" s="32">
         <v>9</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="O27" s="32">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="20">
         <v>13</v>
       </c>
-      <c r="E28" s="28">
+      <c r="E28" s="20">
         <v>21</v>
       </c>
-      <c r="F28" s="28">
+      <c r="F28" s="20">
         <v>16</v>
       </c>
-      <c r="G28" s="28">
+      <c r="G28" s="20">
         <v>9</v>
       </c>
-      <c r="H28" s="28">
+      <c r="H28" s="20">
         <v>11</v>
       </c>
-      <c r="I28" s="28">
+      <c r="I28" s="20">
         <v>10</v>
       </c>
-      <c r="J28" s="28">
+      <c r="J28" s="20">
         <v>7</v>
       </c>
-      <c r="K28" s="28">
+      <c r="K28" s="20">
         <v>20</v>
       </c>
-      <c r="L28" s="28">
+      <c r="L28" s="20">
         <v>16</v>
       </c>
-      <c r="M28" s="28"/>
-      <c r="N28" s="45"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="M28" s="20"/>
+      <c r="N28" s="33"/>
+      <c r="O28" s="33"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D29" s="28">
+      <c r="D29" s="20">
         <v>3</v>
       </c>
-      <c r="E29" s="28">
+      <c r="E29" s="20">
         <v>3</v>
       </c>
-      <c r="F29" s="28">
+      <c r="F29" s="20">
         <v>6</v>
       </c>
-      <c r="G29" s="28">
+      <c r="G29" s="20">
         <v>3</v>
       </c>
-      <c r="H29" s="28">
+      <c r="H29" s="20">
         <v>3</v>
       </c>
-      <c r="I29" s="28">
+      <c r="I29" s="20">
         <v>5</v>
       </c>
-      <c r="J29" s="28">
+      <c r="J29" s="20">
         <v>4</v>
       </c>
-      <c r="K29" s="28">
+      <c r="K29" s="20">
         <v>4</v>
       </c>
-      <c r="L29" s="28">
+      <c r="L29" s="20">
         <v>3</v>
       </c>
-      <c r="M29" s="28"/>
-      <c r="N29" s="45"/>
-    </row>
-    <row r="30" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+      <c r="M29" s="20"/>
+      <c r="N29" s="33"/>
+      <c r="O29" s="33"/>
+    </row>
+    <row r="30" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D30" s="27">
+      <c r="D30" s="19">
         <v>11</v>
       </c>
-      <c r="E30" s="27">
+      <c r="E30" s="19">
         <v>4</v>
       </c>
-      <c r="F30" s="27">
+      <c r="F30" s="19">
         <v>8</v>
       </c>
-      <c r="G30" s="27">
+      <c r="G30" s="19">
         <v>11</v>
       </c>
-      <c r="H30" s="27">
+      <c r="H30" s="19">
         <v>8</v>
       </c>
-      <c r="I30" s="27">
+      <c r="I30" s="19">
         <v>3</v>
       </c>
-      <c r="J30" s="27">
+      <c r="J30" s="19">
         <v>5</v>
       </c>
-      <c r="K30" s="27">
+      <c r="K30" s="19">
         <v>3</v>
       </c>
-      <c r="L30" s="27">
+      <c r="L30" s="19">
         <v>6</v>
       </c>
-      <c r="M30" s="27">
+      <c r="M30" s="19">
         <v>4</v>
       </c>
-      <c r="N30" s="44">
+      <c r="N30" s="32">
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="O30" s="32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="28">
+      <c r="D31" s="20">
         <v>6</v>
       </c>
-      <c r="E31" s="28">
+      <c r="E31" s="20">
         <v>4</v>
       </c>
-      <c r="F31" s="28">
+      <c r="F31" s="20">
         <v>7</v>
       </c>
-      <c r="G31" s="28">
+      <c r="G31" s="20">
         <v>9</v>
       </c>
-      <c r="H31" s="28">
+      <c r="H31" s="20">
         <v>7</v>
       </c>
-      <c r="I31" s="30" t="s">
+      <c r="I31" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="J31" s="28">
+      <c r="J31" s="20">
         <v>5</v>
       </c>
-      <c r="K31" s="28">
+      <c r="K31" s="20">
         <v>2</v>
       </c>
-      <c r="L31" s="28">
+      <c r="L31" s="20">
         <v>5</v>
       </c>
-      <c r="M31" s="28"/>
-      <c r="N31" s="45"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
+      <c r="M31" s="20"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="28">
+      <c r="D32" s="20">
         <v>5</v>
       </c>
-      <c r="E32" s="30" t="s">
+      <c r="E32" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="F32" s="28">
+      <c r="F32" s="20">
         <v>1</v>
       </c>
-      <c r="G32" s="28">
+      <c r="G32" s="20">
         <v>2</v>
       </c>
-      <c r="H32" s="28">
+      <c r="H32" s="20">
         <v>1</v>
       </c>
-      <c r="I32" s="28">
+      <c r="I32" s="20">
         <v>3</v>
       </c>
-      <c r="J32" s="30" t="s">
+      <c r="J32" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="K32" s="28">
+      <c r="K32" s="20">
         <v>1</v>
       </c>
-      <c r="L32" s="28">
+      <c r="L32" s="20">
         <v>1</v>
       </c>
-      <c r="M32" s="28"/>
-      <c r="N32" s="46"/>
-    </row>
-    <row r="33" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
+      <c r="M32" s="20"/>
+      <c r="N32" s="34"/>
+      <c r="O32" s="34"/>
+    </row>
+    <row r="33" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D33" s="27">
+      <c r="D33" s="19">
         <v>101</v>
       </c>
-      <c r="E33" s="27">
+      <c r="E33" s="19">
         <v>103</v>
       </c>
-      <c r="F33" s="27">
+      <c r="F33" s="19">
         <v>95</v>
       </c>
-      <c r="G33" s="27">
+      <c r="G33" s="19">
         <v>89</v>
       </c>
-      <c r="H33" s="27">
+      <c r="H33" s="19">
         <v>72</v>
       </c>
-      <c r="I33" s="27">
+      <c r="I33" s="19">
         <v>49</v>
       </c>
-      <c r="J33" s="27">
+      <c r="J33" s="19">
         <v>52</v>
       </c>
-      <c r="K33" s="27">
+      <c r="K33" s="19">
         <v>60</v>
       </c>
-      <c r="L33" s="27">
+      <c r="L33" s="19">
         <v>62</v>
       </c>
-      <c r="M33" s="27">
+      <c r="M33" s="19">
         <v>35</v>
       </c>
-      <c r="N33" s="44">
+      <c r="N33" s="32">
         <v>27</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
+      <c r="O33" s="32">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D34" s="28">
+      <c r="D34" s="20">
         <v>68</v>
       </c>
-      <c r="E34" s="28">
+      <c r="E34" s="20">
         <v>82</v>
       </c>
-      <c r="F34" s="28">
+      <c r="F34" s="20">
         <v>71</v>
       </c>
-      <c r="G34" s="28">
+      <c r="G34" s="20">
         <v>78</v>
       </c>
-      <c r="H34" s="28">
+      <c r="H34" s="20">
         <v>57</v>
       </c>
-      <c r="I34" s="28">
+      <c r="I34" s="20">
         <v>32</v>
       </c>
-      <c r="J34" s="28">
+      <c r="J34" s="20">
         <v>43</v>
       </c>
-      <c r="K34" s="28">
+      <c r="K34" s="20">
         <v>50</v>
       </c>
-      <c r="L34" s="28">
+      <c r="L34" s="20">
         <v>51</v>
       </c>
-      <c r="M34" s="28"/>
-      <c r="N34" s="45"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="8" t="s">
+      <c r="M34" s="20"/>
+      <c r="N34" s="33"/>
+      <c r="O34" s="33"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D35" s="28">
+      <c r="D35" s="20">
         <v>33</v>
       </c>
-      <c r="E35" s="28">
+      <c r="E35" s="20">
         <v>21</v>
       </c>
-      <c r="F35" s="28">
+      <c r="F35" s="20">
         <v>24</v>
       </c>
-      <c r="G35" s="28">
+      <c r="G35" s="20">
         <v>11</v>
       </c>
-      <c r="H35" s="28">
+      <c r="H35" s="20">
         <v>15</v>
       </c>
-      <c r="I35" s="28">
+      <c r="I35" s="20">
         <v>17</v>
       </c>
-      <c r="J35" s="28">
+      <c r="J35" s="20">
         <v>9</v>
       </c>
-      <c r="K35" s="28">
+      <c r="K35" s="20">
         <v>10</v>
       </c>
-      <c r="L35" s="28">
+      <c r="L35" s="20">
         <v>11</v>
       </c>
-      <c r="M35" s="28"/>
-      <c r="N35" s="45"/>
-    </row>
-    <row r="36" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
+      <c r="M35" s="20"/>
+      <c r="N35" s="33"/>
+      <c r="O35" s="33"/>
+    </row>
+    <row r="36" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D36" s="27">
+      <c r="D36" s="19">
         <v>76</v>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="19">
         <v>67</v>
       </c>
-      <c r="F36" s="27">
+      <c r="F36" s="19">
         <v>55</v>
       </c>
-      <c r="G36" s="27">
+      <c r="G36" s="19">
         <v>69</v>
       </c>
-      <c r="H36" s="27">
+      <c r="H36" s="19">
         <v>44</v>
       </c>
-      <c r="I36" s="27">
+      <c r="I36" s="19">
         <v>32</v>
       </c>
-      <c r="J36" s="27">
+      <c r="J36" s="19">
         <v>30</v>
       </c>
-      <c r="K36" s="27">
+      <c r="K36" s="19">
         <v>40</v>
       </c>
-      <c r="L36" s="27">
+      <c r="L36" s="19">
         <v>48</v>
       </c>
-      <c r="M36" s="27">
+      <c r="M36" s="19">
         <v>19</v>
       </c>
-      <c r="N36" s="44">
+      <c r="N36" s="32">
         <v>21</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="8" t="s">
+      <c r="O36" s="32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D37" s="28">
+      <c r="D37" s="20">
         <v>52</v>
       </c>
-      <c r="E37" s="28">
+      <c r="E37" s="20">
         <v>43</v>
       </c>
-      <c r="F37" s="28">
+      <c r="F37" s="20">
         <v>43</v>
       </c>
-      <c r="G37" s="28">
+      <c r="G37" s="20">
         <v>45</v>
       </c>
-      <c r="H37" s="28">
+      <c r="H37" s="20">
         <v>33</v>
       </c>
-      <c r="I37" s="28">
+      <c r="I37" s="20">
         <v>28</v>
       </c>
-      <c r="J37" s="28">
+      <c r="J37" s="20">
         <v>24</v>
       </c>
-      <c r="K37" s="28">
+      <c r="K37" s="20">
         <v>30</v>
       </c>
-      <c r="L37" s="28">
+      <c r="L37" s="20">
         <v>36</v>
       </c>
-      <c r="M37" s="28"/>
-      <c r="N37" s="45"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
+      <c r="M37" s="20"/>
+      <c r="N37" s="33"/>
+      <c r="O37" s="33"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="28">
+      <c r="D38" s="20">
         <v>24</v>
       </c>
-      <c r="E38" s="28">
+      <c r="E38" s="20">
         <v>24</v>
       </c>
-      <c r="F38" s="28">
+      <c r="F38" s="20">
         <v>12</v>
       </c>
-      <c r="G38" s="28">
+      <c r="G38" s="20">
         <v>24</v>
       </c>
-      <c r="H38" s="28">
+      <c r="H38" s="20">
         <v>11</v>
       </c>
-      <c r="I38" s="28">
+      <c r="I38" s="20">
         <v>4</v>
       </c>
-      <c r="J38" s="28">
+      <c r="J38" s="20">
         <v>6</v>
       </c>
-      <c r="K38" s="28">
+      <c r="K38" s="20">
         <v>10</v>
       </c>
-      <c r="L38" s="28">
+      <c r="L38" s="20">
         <v>12</v>
       </c>
-      <c r="M38" s="28"/>
-      <c r="N38" s="45"/>
-    </row>
-    <row r="39" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+      <c r="M38" s="20"/>
+      <c r="N38" s="33"/>
+      <c r="O38" s="33"/>
+    </row>
+    <row r="39" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D39" s="27">
+      <c r="D39" s="19">
         <v>20</v>
       </c>
-      <c r="E39" s="27">
+      <c r="E39" s="19">
         <v>12</v>
       </c>
-      <c r="F39" s="27">
+      <c r="F39" s="19">
         <v>12</v>
       </c>
-      <c r="G39" s="27">
+      <c r="G39" s="19">
         <v>20</v>
       </c>
-      <c r="H39" s="27">
+      <c r="H39" s="19">
         <v>12</v>
       </c>
-      <c r="I39" s="27">
+      <c r="I39" s="19">
         <v>10</v>
       </c>
-      <c r="J39" s="27">
+      <c r="J39" s="19">
         <v>5</v>
       </c>
-      <c r="K39" s="27">
+      <c r="K39" s="19">
         <v>6</v>
       </c>
-      <c r="L39" s="27">
+      <c r="L39" s="19">
         <v>6</v>
       </c>
-      <c r="M39" s="27">
+      <c r="M39" s="19">
         <v>9</v>
       </c>
-      <c r="N39" s="44">
+      <c r="N39" s="32">
         <v>4</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
+      <c r="O39" s="32">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D40" s="28">
+      <c r="D40" s="20">
         <v>14</v>
       </c>
-      <c r="E40" s="28">
+      <c r="E40" s="20">
         <v>8</v>
       </c>
-      <c r="F40" s="28">
+      <c r="F40" s="20">
         <v>9</v>
       </c>
-      <c r="G40" s="28">
+      <c r="G40" s="20">
         <v>16</v>
       </c>
-      <c r="H40" s="28">
+      <c r="H40" s="20">
         <v>9</v>
       </c>
-      <c r="I40" s="28">
+      <c r="I40" s="20">
         <v>8</v>
       </c>
-      <c r="J40" s="28">
+      <c r="J40" s="20">
         <v>4</v>
       </c>
-      <c r="K40" s="28">
+      <c r="K40" s="20">
         <v>4</v>
       </c>
-      <c r="L40" s="28">
+      <c r="L40" s="20">
         <v>4</v>
       </c>
-      <c r="M40" s="28"/>
-      <c r="N40" s="45"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A41" s="8" t="s">
+      <c r="M40" s="20"/>
+      <c r="N40" s="33"/>
+      <c r="O40" s="33"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="20">
         <v>6</v>
       </c>
-      <c r="E41" s="28">
+      <c r="E41" s="20">
         <v>4</v>
       </c>
-      <c r="F41" s="28">
+      <c r="F41" s="20">
         <v>3</v>
       </c>
-      <c r="G41" s="28">
+      <c r="G41" s="20">
         <v>4</v>
       </c>
-      <c r="H41" s="28">
+      <c r="H41" s="20">
         <v>3</v>
       </c>
-      <c r="I41" s="28">
+      <c r="I41" s="20">
         <v>2</v>
       </c>
-      <c r="J41" s="28">
+      <c r="J41" s="20">
         <v>1</v>
       </c>
-      <c r="K41" s="28">
+      <c r="K41" s="20">
         <v>2</v>
       </c>
-      <c r="L41" s="28">
+      <c r="L41" s="20">
         <v>2</v>
       </c>
-      <c r="M41" s="28"/>
-      <c r="N41" s="45"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+      <c r="M41" s="20"/>
+      <c r="N41" s="33"/>
+      <c r="O41" s="33"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="28"/>
-      <c r="G42" s="28"/>
-      <c r="H42" s="28"/>
-      <c r="I42" s="28"/>
-      <c r="J42" s="28"/>
-      <c r="K42" s="28"/>
-      <c r="L42" s="28"/>
-      <c r="M42" s="28"/>
-      <c r="N42" s="43"/>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A43" s="8" t="s">
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="20"/>
+      <c r="M42" s="20"/>
+      <c r="N42" s="31"/>
+      <c r="O42" s="31"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28">
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="20"/>
+      <c r="K43" s="20"/>
+      <c r="L43" s="20">
         <v>4</v>
       </c>
-      <c r="M43" s="28">
+      <c r="M43" s="20">
         <v>7</v>
       </c>
-      <c r="N43" s="43">
+      <c r="N43" s="31">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A44" s="12" t="s">
+      <c r="O43" s="31">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="C44" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="28"/>
-      <c r="I44" s="28"/>
-      <c r="J44" s="28"/>
-      <c r="K44" s="28"/>
-      <c r="L44" s="28">
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="20"/>
+      <c r="K44" s="20"/>
+      <c r="L44" s="20">
         <v>34</v>
       </c>
-      <c r="M44" s="28">
+      <c r="M44" s="20">
         <v>14</v>
       </c>
-      <c r="N44" s="43">
+      <c r="N44" s="31">
         <v>13</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" s="8" t="s">
+      <c r="O44" s="31">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D45" s="28"/>
-      <c r="E45" s="28"/>
-      <c r="F45" s="28"/>
-      <c r="G45" s="28"/>
-      <c r="H45" s="28"/>
-      <c r="I45" s="28"/>
-      <c r="J45" s="28"/>
-      <c r="K45" s="28"/>
-      <c r="L45" s="28">
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="20"/>
+      <c r="I45" s="20"/>
+      <c r="J45" s="20"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="20">
         <v>109</v>
       </c>
-      <c r="M45" s="28">
+      <c r="M45" s="20">
         <v>65</v>
       </c>
-      <c r="N45" s="43">
+      <c r="N45" s="31">
         <v>50</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A46" s="12" t="s">
+      <c r="O45" s="31">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="28"/>
-      <c r="K46" s="28"/>
-      <c r="L46" s="28">
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
+      <c r="I46" s="20"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
+      <c r="L46" s="20">
         <v>37</v>
       </c>
-      <c r="M46" s="28">
+      <c r="M46" s="20">
         <v>18</v>
       </c>
-      <c r="N46" s="43">
+      <c r="N46" s="31">
         <v>31</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="11" t="s">
+      <c r="O46" s="31">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="31"/>
-      <c r="E47" s="31"/>
-      <c r="F47" s="31"/>
-      <c r="G47" s="31"/>
-      <c r="H47" s="31"/>
-      <c r="I47" s="31"/>
-      <c r="J47" s="31"/>
-      <c r="K47" s="31"/>
-      <c r="L47" s="31">
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23">
         <v>7</v>
       </c>
-      <c r="M47" s="31">
+      <c r="M47" s="23">
         <v>2</v>
       </c>
-      <c r="N47" s="47">
+      <c r="N47" s="35">
         <v>3</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="32" t="s">
+      <c r="O47" s="35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="32" t="s">
+      <c r="B48" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="32" t="s">
+      <c r="C48" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="N48" s="39"/>
+      <c r="N48" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>